<commit_message>
fix: Ajuste a 2 decimales y corrección de mapa
</commit_message>
<xml_diff>
--- a/datasets/Ranking PE VCEyEC Distritos.xlsx
+++ b/datasets/Ranking PE VCEyEC Distritos.xlsx
@@ -5,16 +5,19 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\INE\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\INE\Documents\reductor_dias\datasets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{9BA3FCB7-0005-49EB-84A7-08C3539A9561}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{77619903-2BF7-46DE-A7A1-EA089A69CBA1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{F3830E03-ADB1-4D4C-911D-3B58AE903CE7}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="4" r:id="rId1"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Hoja1!$A$1:$G$299</definedName>
+  </definedNames>
   <calcPr calcId="191028"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -405,17 +408,17 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="2" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="2" xfId="0" quotePrefix="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" quotePrefix="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2213,7 +2216,7 @@
         <v>85</v>
       </c>
       <c r="D64" s="12" t="s">
-        <v>10</v>
+        <v>21</v>
       </c>
       <c r="E64" s="4" t="s">
         <v>6</v>
@@ -7631,6 +7634,7 @@
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:G299" xr:uid="{D2177327-B67A-4242-8318-7AC97FFA32A3}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>